<commit_message>
updating to remove useless things
</commit_message>
<xml_diff>
--- a/docs/handover/04-RBAC/RBAC_MATRIX.xlsx
+++ b/docs/handover/04-RBAC/RBAC_MATRIX.xlsx
@@ -486,7 +486,7 @@
         <v>Full portal access including privileged Super Admin controls</v>
       </c>
       <c r="D6">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -512,7 +512,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -723,7 +723,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>manage_users</v>
+        <v>page_spare_loan_check</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -732,13 +732,13 @@
         <v/>
       </c>
       <c r="D10" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="E10" t="str">
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -746,7 +746,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>manage_roles</v>
+        <v>manage_users</v>
       </c>
       <c r="B11" t="str">
         <v/>
@@ -769,7 +769,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>manage_users</v>
+        <v>manage_roles</v>
       </c>
       <c r="B12" t="str">
         <v/>
@@ -815,7 +815,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>super_admin</v>
+        <v>manage_users</v>
       </c>
       <c r="B14" t="str">
         <v/>
@@ -824,7 +824,7 @@
         <v/>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -838,7 +838,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>page_mis_email_settings</v>
+        <v>super_admin</v>
       </c>
       <c r="B15" t="str">
         <v/>
@@ -861,7 +861,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>page_mis_email_routing</v>
+        <v>page_mis_email_settings</v>
       </c>
       <c r="B16" t="str">
         <v/>
@@ -884,7 +884,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>page_major_repair_alerts</v>
+        <v>page_mis_email_routing</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -907,7 +907,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>page_cancelled_call_alerts</v>
+        <v>page_major_repair_alerts</v>
       </c>
       <c r="B18" t="str">
         <v/>
@@ -916,7 +916,7 @@
         <v/>
       </c>
       <c r="D18" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -930,7 +930,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>page_performance_insights</v>
+        <v>page_cancelled_call_alerts</v>
       </c>
       <c r="B19" t="str">
         <v/>
@@ -953,30 +953,30 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>tab_mis_summary</v>
+        <v>page_performance_insights</v>
       </c>
       <c r="B20" t="str">
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="D20" t="str">
         <v>Y</v>
       </c>
       <c r="E20" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="F20" t="str">
         <v>Y</v>
       </c>
       <c r="G20" t="str">
-        <v>Y</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>tab_mis_register</v>
+        <v>tab_mis_summary</v>
       </c>
       <c r="B21" t="str">
         <v/>
@@ -999,7 +999,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>tab_mis_accounts</v>
+        <v>tab_mis_register</v>
       </c>
       <c r="B22" t="str">
         <v/>
@@ -1022,7 +1022,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>tab_mis_client_import</v>
+        <v>tab_mis_accounts</v>
       </c>
       <c r="B23" t="str">
         <v/>
@@ -1034,7 +1034,7 @@
         <v>Y</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="F23" t="str">
         <v>Y</v>
@@ -1045,7 +1045,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>tab_mis_bd_mis_summary</v>
+        <v>tab_mis_client_import</v>
       </c>
       <c r="B24" t="str">
         <v/>
@@ -1068,16 +1068,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>tab_mis_deployment_completion</v>
+        <v>tab_mis_bd_mis_summary</v>
       </c>
       <c r="B25" t="str">
         <v/>
       </c>
       <c r="C25" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>Y</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -1086,12 +1086,12 @@
         <v>Y</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>Y</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>view_all_offices</v>
+        <v>tab_mis_deployment_completion</v>
       </c>
       <c r="B26" t="str">
         <v/>
@@ -1114,16 +1114,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>mis_client_import_upload</v>
+        <v>view_all_offices</v>
       </c>
       <c r="B27" t="str">
         <v/>
       </c>
       <c r="C27" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="D27" t="str">
-        <v>Y</v>
+        <v/>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -1132,42 +1132,65 @@
         <v>Y</v>
       </c>
       <c r="G27" t="str">
-        <v>Y</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>mis_client_import_upload</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>Y</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Y</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>mis_client_import_delete</v>
       </c>
-      <c r="B28" t="str">
-        <v/>
-      </c>
-      <c r="C28" t="str">
-        <v>Y</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Y</v>
-      </c>
-      <c r="E28" t="str">
-        <v/>
-      </c>
-      <c r="F28" t="str">
-        <v>Y</v>
-      </c>
-      <c r="G28" t="str">
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>Y</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Y</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v>Y</v>
+      </c>
+      <c r="G29" t="str">
         <v>Y</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B90"/>
+  <dimension ref="A1:B86"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1758,39 +1781,39 @@
         <v>Super Admin</v>
       </c>
       <c r="B74" t="str">
-        <v>view_mis_accounts</v>
+        <v>view_reports</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Super Admin</v>
+        <v>View Summary</v>
       </c>
       <c r="B75" t="str">
-        <v>view_mis_register</v>
+        <v>mis_client_import_delete</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Super Admin</v>
+        <v>View Summary</v>
       </c>
       <c r="B76" t="str">
-        <v>view_mis_summary</v>
+        <v>mis_client_import_upload</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Super Admin</v>
+        <v>View Summary</v>
       </c>
       <c r="B77" t="str">
-        <v>view_reports</v>
+        <v>mis_email_send</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Super Admin</v>
+        <v>View Summary</v>
       </c>
       <c r="B78" t="str">
-        <v>view_summary</v>
+        <v>page_athena_reconciliation</v>
       </c>
     </row>
     <row r="79">
@@ -1798,7 +1821,7 @@
         <v>View Summary</v>
       </c>
       <c r="B79" t="str">
-        <v>mis_client_import_delete</v>
+        <v>page_cancelled_calls</v>
       </c>
     </row>
     <row r="80">
@@ -1806,7 +1829,7 @@
         <v>View Summary</v>
       </c>
       <c r="B80" t="str">
-        <v>mis_client_import_upload</v>
+        <v>page_mis_reports</v>
       </c>
     </row>
     <row r="81">
@@ -1814,7 +1837,7 @@
         <v>View Summary</v>
       </c>
       <c r="B81" t="str">
-        <v>mis_email_send</v>
+        <v>page_serial_audit</v>
       </c>
     </row>
     <row r="82">
@@ -1822,7 +1845,7 @@
         <v>View Summary</v>
       </c>
       <c r="B82" t="str">
-        <v>page_athena_reconciliation</v>
+        <v>tab_mis_accounts</v>
       </c>
     </row>
     <row r="83">
@@ -1830,7 +1853,7 @@
         <v>View Summary</v>
       </c>
       <c r="B83" t="str">
-        <v>page_cancelled_calls</v>
+        <v>tab_mis_bd_mis_summary</v>
       </c>
     </row>
     <row r="84">
@@ -1838,7 +1861,7 @@
         <v>View Summary</v>
       </c>
       <c r="B84" t="str">
-        <v>page_mis_reports</v>
+        <v>tab_mis_client_import</v>
       </c>
     </row>
     <row r="85">
@@ -1846,7 +1869,7 @@
         <v>View Summary</v>
       </c>
       <c r="B85" t="str">
-        <v>page_serial_audit</v>
+        <v>tab_mis_register</v>
       </c>
     </row>
     <row r="86">
@@ -1854,51 +1877,19 @@
         <v>View Summary</v>
       </c>
       <c r="B86" t="str">
-        <v>tab_mis_accounts</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="str">
-        <v>View Summary</v>
-      </c>
-      <c r="B87" t="str">
-        <v>tab_mis_bd_mis_summary</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="str">
-        <v>View Summary</v>
-      </c>
-      <c r="B88" t="str">
-        <v>tab_mis_client_import</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="str">
-        <v>View Summary</v>
-      </c>
-      <c r="B89" t="str">
-        <v>tab_mis_register</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="str">
-        <v>View Summary</v>
-      </c>
-      <c r="B90" t="str">
         <v>tab_mis_summary</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B90"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B86"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2055,16 +2046,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>manage_users</v>
+        <v>page_spare_loan_check</v>
       </c>
       <c r="B10" t="str">
-        <v>User Management</v>
+        <v>Spare Loan Check</v>
       </c>
       <c r="C10" t="str">
-        <v>/admin/users</v>
+        <v>/report/spare-loan-check</v>
       </c>
       <c r="D10" t="str">
-        <v>Administration</v>
+        <v>Reports</v>
       </c>
       <c r="E10" t="str">
         <v>yes</v>
@@ -2072,13 +2063,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>manage_roles</v>
+        <v>manage_users</v>
       </c>
       <c r="B11" t="str">
-        <v>Roles &amp; Access</v>
+        <v>User Management</v>
       </c>
       <c r="C11" t="str">
-        <v>/admin/roles</v>
+        <v>/admin/users</v>
       </c>
       <c r="D11" t="str">
         <v>Administration</v>
@@ -2089,19 +2080,19 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>manage_users</v>
+        <v>manage_roles</v>
       </c>
       <c r="B12" t="str">
-        <v>Read-model sync</v>
+        <v>Roles &amp; Access</v>
       </c>
       <c r="C12" t="str">
-        <v>/admin/sync</v>
+        <v>/admin/roles</v>
       </c>
       <c r="D12" t="str">
         <v>Administration</v>
       </c>
       <c r="E12" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="13">
@@ -2109,10 +2100,10 @@
         <v>manage_users</v>
       </c>
       <c r="B13" t="str">
-        <v>Service call activity</v>
+        <v>Read-model sync</v>
       </c>
       <c r="C13" t="str">
-        <v>/admin/attendance</v>
+        <v>/admin/sync</v>
       </c>
       <c r="D13" t="str">
         <v>Administration</v>
@@ -2123,13 +2114,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>super_admin</v>
+        <v>manage_users</v>
       </c>
       <c r="B14" t="str">
-        <v>VPS Cron</v>
+        <v>Service call activity</v>
       </c>
       <c r="C14" t="str">
-        <v>/admin/vps-cron</v>
+        <v>/admin/attendance</v>
       </c>
       <c r="D14" t="str">
         <v>Administration</v>
@@ -2140,47 +2131,47 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>page_mis_email_settings</v>
+        <v>super_admin</v>
       </c>
       <c r="B15" t="str">
-        <v>Mail &amp; Alerts</v>
+        <v>VPS Cron</v>
       </c>
       <c r="C15" t="str">
-        <v>/admin/mis-email-settings</v>
+        <v>/admin/vps-cron</v>
       </c>
       <c r="D15" t="str">
         <v>Administration</v>
       </c>
       <c r="E15" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>page_mis_email_routing</v>
+        <v>page_mis_email_settings</v>
       </c>
       <c r="B16" t="str">
-        <v>MIS Email Routing</v>
+        <v>Mail &amp; Alerts</v>
       </c>
       <c r="C16" t="str">
-        <v>/admin/mis-email-routing</v>
+        <v>/admin/mis-email-settings</v>
       </c>
       <c r="D16" t="str">
         <v>Administration</v>
       </c>
       <c r="E16" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>page_major_repair_alerts</v>
+        <v>page_mis_email_routing</v>
       </c>
       <c r="B17" t="str">
-        <v>Major Repair Alerts</v>
+        <v>MIS Email Routing</v>
       </c>
       <c r="C17" t="str">
-        <v>/admin/major-repair-alerts</v>
+        <v>/admin/mis-email-routing</v>
       </c>
       <c r="D17" t="str">
         <v>Administration</v>
@@ -2191,13 +2182,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>page_cancelled_call_alerts</v>
+        <v>page_major_repair_alerts</v>
       </c>
       <c r="B18" t="str">
-        <v>Cancelled Call Digests</v>
+        <v>Major Repair Alerts</v>
       </c>
       <c r="C18" t="str">
-        <v>/admin/cancelled-call-alerts</v>
+        <v>/admin/major-repair-alerts</v>
       </c>
       <c r="D18" t="str">
         <v>Administration</v>
@@ -2208,24 +2199,41 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>page_performance_insights</v>
+        <v>page_cancelled_call_alerts</v>
       </c>
       <c r="B19" t="str">
-        <v>Performance Insights</v>
+        <v>Cancelled Call Digests</v>
       </c>
       <c r="C19" t="str">
-        <v>/admin/performance-insights</v>
+        <v>/admin/cancelled-call-alerts</v>
       </c>
       <c r="D19" t="str">
         <v>Administration</v>
       </c>
       <c r="E19" t="str">
+        <v>no</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>page_performance_insights</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Performance Insights</v>
+      </c>
+      <c r="C20" t="str">
+        <v>/admin/performance-insights</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="E20" t="str">
         <v>yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2387,7 +2395,7 @@
         <v>Exported</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-02T05:51:55Z</v>
+        <v>2026-09-07T09:19:58Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>